<commit_message>
Nuevo caso individual (2026-06-30T04:08:08)
</commit_message>
<xml_diff>
--- a/data/casos_ingresados.xlsx
+++ b/data/casos_ingresados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,72 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>2026-06-30T04:03:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>UCO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H. Penco-Lirquén</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sonda vesical foley</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>B.I.a.e2.Síntomas irritativos vesicales (tenesmo vesical, urgencia miccional, polaquiuria, disuria, dolor suprapúbico)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>B.I.c.e1.Cultivo de orina con no más de dos microorganismos, en el que al menos uno de ellos tiene recuento de más de 100.000 UFC/ml</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>IAAS</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-06-30T04:08:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nuevo caso individual (2026-06-30T05:35:51)
</commit_message>
<xml_diff>
--- a/data/casos_ingresados.xlsx
+++ b/data/casos_ingresados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -617,6 +617,72 @@
       <c r="N3" t="inlineStr">
         <is>
           <t>2026-06-30T04:08:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sala de cuidados intermedios</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Emergencia</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Catéter epicutáneo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>C.II.a.e2.Sensibilidad o dolor en la zona de la incisión quirúrgica</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>NO IAAS</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-06-30T05:35:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nuevo caso individual (2026-06-30T05:36:23)
</commit_message>
<xml_diff>
--- a/data/casos_ingresados.xlsx
+++ b/data/casos_ingresados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,6 +683,72 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>2026-06-30T05:35:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sala de cuidados intermedios</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Emergencia</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Catéter epicutáneo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>C.II.a.e2.Sensibilidad o dolor en la zona de la incisión quirúrgica</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>C.I.a.e1.Presencia de pus (exudado purulento) en el sitio de incisión quirúrgica, incluido el sitio de la salida de drenaje por contrabertura, con o sin cultivos positivos</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sin hallazgos IAAS</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NO IAAS</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-06-30T05:36:23</t>
         </is>
       </c>
     </row>

</xml_diff>